<commit_message>
Actualiza dashboard con corte del 18 de agosto
</commit_message>
<xml_diff>
--- a/Dashboard_Matriculas_CUC_2026-2.xlsx
+++ b/Dashboard_Matriculas_CUC_2026-2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen ejecutivo" sheetId="1" r:id="R063726398cde4ad2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado por programa" sheetId="2" r:id="R9a66a69c386a4887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrícula académica" sheetId="3" r:id="R9285fff404dc4971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embudo de admisiones" sheetId="4" r:id="Rf522cdaf76a44e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen ejecutivo" sheetId="1" r:id="R7863787f1a794e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado por programa" sheetId="2" r:id="R9e678147996749c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrícula académica" sheetId="3" r:id="Ra09e180092844861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embudo de admisiones" sheetId="4" r:id="R9749fc450c424dc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -459,7 +459,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Corte institucional del 12 de agosto de 2026 · Cumplimiento basado en matrícula financiera</x:v>
+        <x:v>Corte institucional del 18 de agosto de 2026 · Cumplimiento basado en matrícula financiera</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -494,7 +494,7 @@
       </x:c>
       <x:c r="E5" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!B5:B26)</x:f>
-        <x:v>985</x:v>
+        <x:v>991</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -503,14 +503,14 @@
       </x:c>
       <x:c r="B6" s="13" t="n">
         <x:f>SUM('Consolidado por programa'!D5:D31)</x:f>
-        <x:v>469</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
         <x:v>Inscritos</x:v>
       </x:c>
       <x:c r="E6" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!C5:C26)</x:f>
-        <x:v>665</x:v>
+        <x:v>672</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -518,15 +518,15 @@
         <x:v>Cumplimiento financiero</x:v>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:f>B6/B5</x:f>
-        <x:v>0.8330373001776199</x:v>
+        <x:f>IF(B5=0,0,B6/B5)</x:f>
+        <x:v>0.8650088809946714</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
         <x:v>Admitidos</x:v>
       </x:c>
       <x:c r="E7" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!D5:D26)</x:f>
-        <x:v>621</x:v>
+        <x:v>624</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -535,14 +535,14 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>MAX(B5-B6,0)</x:f>
-        <x:v>94</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
         <x:v>Por admitir</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
-        <x:f>363</x:f>
-        <x:v>363</x:v>
+        <x:f>MAX(E5-E7-E9,0)</x:f>
+        <x:v>366</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -551,19 +551,18 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>SUM('Consolidado por programa'!E5:E31)</x:f>
-        <x:v>538</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Rechazados</x:v>
       </x:c>
       <x:c r="E9" s="13" t="n">
-        <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18" t="str">
-        <x:v>Lectura: 469 estudiantes han completado la matrícula financiera. Las 538 matrículas académicas representan 69 estudiantes de diferencia respecto al pago y funcionan como indicador complementario de proximidad.</x:v>
+        <x:v>Lectura: 487 estudiantes han completado la matrícula financiera. Las 568 matrículas académicas de primer nivel representan 81 estudiantes de diferencia respecto al pago y funcionan como indicador complementario de proximidad.</x:v>
       </x:c>
       <x:c r="B11" s="18"/>
       <x:c r="C11" s="18"/>
@@ -621,7 +620,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Metas, matrícula financiera y matrícula académica · Periodo 2026-2</x:v>
+        <x:v>Metas, matrícula financiera y matrícula académica · Periodo 2026-2 · Corte 18 de agosto de 2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -690,11 +689,11 @@
         <x:f>IF(OR(B5=0,D5=""),"",MAX(B5-D5,0))</x:f>
       </x:c>
       <x:c r="I5" s="27" t="str">
-        <x:f>IF(B5=0,"Sin meta",IF(D5="","Sin dato financiero",IF(D5&gt;B5,"Superada",IF(D5=B5,"Cumplida",IF(G5&gt;=0.8,"Cerca",IF(G5&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B5=0,"Sin meta",IF(D5="","Sin dato financiero",IF(D5&gt;B5,"Superada",IF(D5=B5,"Cumplida",IF(D5/B5&gt;=0.8,"Cerca",IF(D5/B5&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J5" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -727,11 +726,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="27" t="str">
-        <x:f>IF(B6=0,"Sin meta",IF(D6="","Sin dato financiero",IF(D6&gt;B6,"Superada",IF(D6=B6,"Cumplida",IF(G6&gt;=0.8,"Cerca",IF(G6&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B6=0,"Sin meta",IF(D6="","Sin dato financiero",IF(D6&gt;B6,"Superada",IF(D6=B6,"Cumplida",IF(D6/B6&gt;=0.8,"Cerca",IF(D6/B6&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Cumplida</x:v>
       </x:c>
       <x:c r="J6" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -759,11 +758,11 @@
         <x:f>IF(OR(B7=0,D7=""),"",MAX(B7-D7,0))</x:f>
       </x:c>
       <x:c r="I7" s="27" t="str">
-        <x:f>IF(B7=0,"Sin meta",IF(D7="","Sin dato financiero",IF(D7&gt;B7,"Superada",IF(D7=B7,"Cumplida",IF(G7&gt;=0.8,"Cerca",IF(G7&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B7=0,"Sin meta",IF(D7="","Sin dato financiero",IF(D7&gt;B7,"Superada",IF(D7=B7,"Cumplida",IF(D7/B7&gt;=0.8,"Cerca",IF(D7/B7&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J7" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -781,11 +780,11 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E8" s="25" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F8" s="25" t="n">
         <x:f>IF(D8="","",E8-D8)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="26" t="n">
         <x:f>IF(OR(B8=0,D8=""),"",D8/B8)</x:f>
@@ -796,11 +795,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
-        <x:f>IF(B8=0,"Sin meta",IF(D8="","Sin dato financiero",IF(D8&gt;B8,"Superada",IF(D8=B8,"Cumplida",IF(G8&gt;=0.8,"Cerca",IF(G8&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B8=0,"Sin meta",IF(D8="","Sin dato financiero",IF(D8&gt;B8,"Superada",IF(D8=B8,"Cumplida",IF(D8/B8&gt;=0.8,"Cerca",IF(D8/B8&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J8" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -815,29 +814,29 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D9" s="25" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E9" s="25" t="n">
-        <x:v>29</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>IF(D9="","",E9-D9)</x:f>
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G9" s="26" t="n">
         <x:f>IF(OR(B9=0,D9=""),"",D9/B9)</x:f>
-        <x:v>0.5277777777777778</x:v>
+        <x:v>0.5555555555555556</x:v>
       </x:c>
       <x:c r="H9" s="25" t="n">
         <x:f>IF(OR(B9=0,D9=""),"",MAX(B9-D9,0))</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I9" s="27" t="str">
-        <x:f>IF(B9=0,"Sin meta",IF(D9="","Sin dato financiero",IF(D9&gt;B9,"Superada",IF(D9=B9,"Cumplida",IF(G9&gt;=0.8,"Cerca",IF(G9&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B9=0,"Sin meta",IF(D9="","Sin dato financiero",IF(D9&gt;B9,"Superada",IF(D9=B9,"Cumplida",IF(D9/B9&gt;=0.8,"Cerca",IF(D9/B9&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J9" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -865,11 +864,11 @@
         <x:f>IF(OR(B10=0,D10=""),"",MAX(B10-D10,0))</x:f>
       </x:c>
       <x:c r="I10" s="27" t="str">
-        <x:f>IF(B10=0,"Sin meta",IF(D10="","Sin dato financiero",IF(D10&gt;B10,"Superada",IF(D10=B10,"Cumplida",IF(G10&gt;=0.8,"Cerca",IF(G10&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B10=0,"Sin meta",IF(D10="","Sin dato financiero",IF(D10&gt;B10,"Superada",IF(D10=B10,"Cumplida",IF(D10/B10&gt;=0.8,"Cerca",IF(D10/B10&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J10" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -884,10 +883,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D11" s="25" t="n">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E11" s="25" t="n">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F11" s="25" t="n">
         <x:f>IF(D11="","",E11-D11)</x:f>
@@ -895,18 +894,18 @@
       </x:c>
       <x:c r="G11" s="26" t="n">
         <x:f>IF(OR(B11=0,D11=""),"",D11/B11)</x:f>
-        <x:v>1.15</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="H11" s="25" t="n">
         <x:f>IF(OR(B11=0,D11=""),"",MAX(B11-D11,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="27" t="str">
-        <x:f>IF(B11=0,"Sin meta",IF(D11="","Sin dato financiero",IF(D11&gt;B11,"Superada",IF(D11=B11,"Cumplida",IF(G11&gt;=0.8,"Cerca",IF(G11&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B11=0,"Sin meta",IF(D11="","Sin dato financiero",IF(D11&gt;B11,"Superada",IF(D11=B11,"Cumplida",IF(D11/B11&gt;=0.8,"Cerca",IF(D11/B11&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J11" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -921,10 +920,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D12" s="25" t="n">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E12" s="25" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F12" s="25" t="n">
         <x:f>IF(D12="","",E12-D12)</x:f>
@@ -932,18 +931,18 @@
       </x:c>
       <x:c r="G12" s="26" t="n">
         <x:f>IF(OR(B12=0,D12=""),"",D12/B12)</x:f>
-        <x:v>1.3181818181818181</x:v>
+        <x:v>1.3636363636363635</x:v>
       </x:c>
       <x:c r="H12" s="25" t="n">
         <x:f>IF(OR(B12=0,D12=""),"",MAX(B12-D12,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="27" t="str">
-        <x:f>IF(B12=0,"Sin meta",IF(D12="","Sin dato financiero",IF(D12&gt;B12,"Superada",IF(D12=B12,"Cumplida",IF(G12&gt;=0.8,"Cerca",IF(G12&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B12=0,"Sin meta",IF(D12="","Sin dato financiero",IF(D12&gt;B12,"Superada",IF(D12=B12,"Cumplida",IF(D12/B12&gt;=0.8,"Cerca",IF(D12/B12&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J12" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -958,10 +957,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D13" s="25" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E13" s="25" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F13" s="25" t="n">
         <x:f>IF(D13="","",E13-D13)</x:f>
@@ -969,18 +968,18 @@
       </x:c>
       <x:c r="G13" s="26" t="n">
         <x:f>IF(OR(B13=0,D13=""),"",D13/B13)</x:f>
-        <x:v>1</x:v>
+        <x:v>1.125</x:v>
       </x:c>
       <x:c r="H13" s="25" t="n">
         <x:f>IF(OR(B13=0,D13=""),"",MAX(B13-D13,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="27" t="str">
-        <x:f>IF(B13=0,"Sin meta",IF(D13="","Sin dato financiero",IF(D13&gt;B13,"Superada",IF(D13=B13,"Cumplida",IF(G13&gt;=0.8,"Cerca",IF(G13&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
-        <x:v>Cumplida</x:v>
+        <x:f>IF(B13=0,"Sin meta",IF(D13="","Sin dato financiero",IF(D13&gt;B13,"Superada",IF(D13=B13,"Cumplida",IF(D13/B13&gt;=0.8,"Cerca",IF(D13/B13&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:v>Superada</x:v>
       </x:c>
       <x:c r="J13" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -995,29 +994,29 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D14" s="25" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E14" s="25" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F14" s="25" t="n">
         <x:f>IF(D14="","",E14-D14)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G14" s="26" t="n">
         <x:f>IF(OR(B14=0,D14=""),"",D14/B14)</x:f>
-        <x:v>0.45714285714285713</x:v>
+        <x:v>0.4857142857142857</x:v>
       </x:c>
       <x:c r="H14" s="25" t="n">
         <x:f>IF(OR(B14=0,D14=""),"",MAX(B14-D14,0))</x:f>
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="I14" s="27" t="str">
-        <x:f>IF(B14=0,"Sin meta",IF(D14="","Sin dato financiero",IF(D14&gt;B14,"Superada",IF(D14=B14,"Cumplida",IF(G14&gt;=0.8,"Cerca",IF(G14&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B14=0,"Sin meta",IF(D14="","Sin dato financiero",IF(D14&gt;B14,"Superada",IF(D14=B14,"Cumplida",IF(D14/B14&gt;=0.8,"Cerca",IF(D14/B14&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Rezagada</x:v>
       </x:c>
       <x:c r="J14" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1032,10 +1031,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D15" s="25" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E15" s="25" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F15" s="25" t="n">
         <x:f>IF(D15="","",E15-D15)</x:f>
@@ -1043,18 +1042,18 @@
       </x:c>
       <x:c r="G15" s="26" t="n">
         <x:f>IF(OR(B15=0,D15=""),"",D15/B15)</x:f>
-        <x:v>1</x:v>
+        <x:v>1.1428571428571428</x:v>
       </x:c>
       <x:c r="H15" s="25" t="n">
         <x:f>IF(OR(B15=0,D15=""),"",MAX(B15-D15,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="27" t="str">
-        <x:f>IF(B15=0,"Sin meta",IF(D15="","Sin dato financiero",IF(D15&gt;B15,"Superada",IF(D15=B15,"Cumplida",IF(G15&gt;=0.8,"Cerca",IF(G15&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
-        <x:v>Cumplida</x:v>
+        <x:f>IF(B15=0,"Sin meta",IF(D15="","Sin dato financiero",IF(D15&gt;B15,"Superada",IF(D15=B15,"Cumplida",IF(D15/B15&gt;=0.8,"Cerca",IF(D15/B15&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:v>Superada</x:v>
       </x:c>
       <x:c r="J15" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1087,11 +1086,11 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="I16" s="27" t="str">
-        <x:f>IF(B16=0,"Sin meta",IF(D16="","Sin dato financiero",IF(D16&gt;B16,"Superada",IF(D16=B16,"Cumplida",IF(G16&gt;=0.8,"Cerca",IF(G16&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B16=0,"Sin meta",IF(D16="","Sin dato financiero",IF(D16&gt;B16,"Superada",IF(D16=B16,"Cumplida",IF(D16/B16&gt;=0.8,"Cerca",IF(D16/B16&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J16" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1106,29 +1105,29 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D17" s="25" t="n">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E17" s="25" t="n">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F17" s="25" t="n">
         <x:f>IF(D17="","",E17-D17)</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G17" s="26" t="n">
         <x:f>IF(OR(B17=0,D17=""),"",D17/B17)</x:f>
-        <x:v>0.7083333333333334</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="H17" s="25" t="n">
         <x:f>IF(OR(B17=0,D17=""),"",MAX(B17-D17,0))</x:f>
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I17" s="27" t="str">
-        <x:f>IF(B17=0,"Sin meta",IF(D17="","Sin dato financiero",IF(D17&gt;B17,"Superada",IF(D17=B17,"Cumplida",IF(G17&gt;=0.8,"Cerca",IF(G17&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B17=0,"Sin meta",IF(D17="","Sin dato financiero",IF(D17&gt;B17,"Superada",IF(D17=B17,"Cumplida",IF(D17/B17&gt;=0.8,"Cerca",IF(D17/B17&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J17" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1143,29 +1142,29 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D18" s="25" t="n">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E18" s="25" t="n">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="F18" s="25" t="n">
         <x:f>IF(D18="","",E18-D18)</x:f>
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G18" s="26" t="n">
         <x:f>IF(OR(B18=0,D18=""),"",D18/B18)</x:f>
-        <x:v>0.6</x:v>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="H18" s="25" t="n">
         <x:f>IF(OR(B18=0,D18=""),"",MAX(B18-D18,0))</x:f>
-        <x:v>24</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I18" s="27" t="str">
-        <x:f>IF(B18=0,"Sin meta",IF(D18="","Sin dato financiero",IF(D18&gt;B18,"Superada",IF(D18=B18,"Cumplida",IF(G18&gt;=0.8,"Cerca",IF(G18&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B18=0,"Sin meta",IF(D18="","Sin dato financiero",IF(D18&gt;B18,"Superada",IF(D18=B18,"Cumplida",IF(D18/B18&gt;=0.8,"Cerca",IF(D18/B18&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J18" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1183,11 +1182,11 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E19" s="25" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F19" s="25" t="n">
         <x:f>IF(D19="","",E19-D19)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G19" s="26" t="n">
         <x:f>IF(OR(B19=0,D19=""),"",D19/B19)</x:f>
@@ -1198,11 +1197,11 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="I19" s="27" t="str">
-        <x:f>IF(B19=0,"Sin meta",IF(D19="","Sin dato financiero",IF(D19&gt;B19,"Superada",IF(D19=B19,"Cumplida",IF(G19&gt;=0.8,"Cerca",IF(G19&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B19=0,"Sin meta",IF(D19="","Sin dato financiero",IF(D19&gt;B19,"Superada",IF(D19=B19,"Cumplida",IF(D19/B19&gt;=0.8,"Cerca",IF(D19/B19&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J19" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1235,11 +1234,11 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="I20" s="27" t="str">
-        <x:f>IF(B20=0,"Sin meta",IF(D20="","Sin dato financiero",IF(D20&gt;B20,"Superada",IF(D20=B20,"Cumplida",IF(G20&gt;=0.8,"Cerca",IF(G20&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B20=0,"Sin meta",IF(D20="","Sin dato financiero",IF(D20&gt;B20,"Superada",IF(D20=B20,"Cumplida",IF(D20/B20&gt;=0.8,"Cerca",IF(D20/B20&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J20" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1272,11 +1271,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I21" s="27" t="str">
-        <x:f>IF(B21=0,"Sin meta",IF(D21="","Sin dato financiero",IF(D21&gt;B21,"Superada",IF(D21=B21,"Cumplida",IF(G21&gt;=0.8,"Cerca",IF(G21&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B21=0,"Sin meta",IF(D21="","Sin dato financiero",IF(D21&gt;B21,"Superada",IF(D21=B21,"Cumplida",IF(D21/B21&gt;=0.8,"Cerca",IF(D21/B21&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Cerca</x:v>
       </x:c>
       <x:c r="J21" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1291,10 +1290,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D22" s="25" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E22" s="25" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F22" s="25" t="n">
         <x:f>IF(D22="","",E22-D22)</x:f>
@@ -1302,18 +1301,18 @@
       </x:c>
       <x:c r="G22" s="26" t="n">
         <x:f>IF(OR(B22=0,D22=""),"",D22/B22)</x:f>
-        <x:v>0.34782608695652173</x:v>
+        <x:v>0.391304347826087</x:v>
       </x:c>
       <x:c r="H22" s="25" t="n">
         <x:f>IF(OR(B22=0,D22=""),"",MAX(B22-D22,0))</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="I22" s="27" t="str">
-        <x:f>IF(B22=0,"Sin meta",IF(D22="","Sin dato financiero",IF(D22&gt;B22,"Superada",IF(D22=B22,"Cumplida",IF(G22&gt;=0.8,"Cerca",IF(G22&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B22=0,"Sin meta",IF(D22="","Sin dato financiero",IF(D22&gt;B22,"Superada",IF(D22=B22,"Cumplida",IF(D22/B22&gt;=0.8,"Cerca",IF(D22/B22&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Rezagada</x:v>
       </x:c>
       <x:c r="J22" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1341,11 +1340,11 @@
         <x:f>IF(OR(B23=0,D23=""),"",MAX(B23-D23,0))</x:f>
       </x:c>
       <x:c r="I23" s="27" t="str">
-        <x:f>IF(B23=0,"Sin meta",IF(D23="","Sin dato financiero",IF(D23&gt;B23,"Superada",IF(D23=B23,"Cumplida",IF(G23&gt;=0.8,"Cerca",IF(G23&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B23=0,"Sin meta",IF(D23="","Sin dato financiero",IF(D23&gt;B23,"Superada",IF(D23=B23,"Cumplida",IF(D23/B23&gt;=0.8,"Cerca",IF(D23/B23&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J23" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1360,10 +1359,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D24" s="25" t="n">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E24" s="25" t="n">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F24" s="25" t="n">
         <x:f>IF(D24="","",E24-D24)</x:f>
@@ -1371,18 +1370,18 @@
       </x:c>
       <x:c r="G24" s="26" t="n">
         <x:f>IF(OR(B24=0,D24=""),"",D24/B24)</x:f>
-        <x:v>1.2962962962962963</x:v>
+        <x:v>1.3333333333333333</x:v>
       </x:c>
       <x:c r="H24" s="25" t="n">
         <x:f>IF(OR(B24=0,D24=""),"",MAX(B24-D24,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I24" s="27" t="str">
-        <x:f>IF(B24=0,"Sin meta",IF(D24="","Sin dato financiero",IF(D24&gt;B24,"Superada",IF(D24=B24,"Cumplida",IF(G24&gt;=0.8,"Cerca",IF(G24&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B24=0,"Sin meta",IF(D24="","Sin dato financiero",IF(D24&gt;B24,"Superada",IF(D24=B24,"Cumplida",IF(D24/B24&gt;=0.8,"Cerca",IF(D24/B24&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J24" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1397,29 +1396,29 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D25" s="25" t="n">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E25" s="25" t="n">
-        <x:v>51</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="F25" s="25" t="n">
         <x:f>IF(D25="","",E25-D25)</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G25" s="26" t="n">
         <x:f>IF(OR(B25=0,D25=""),"",D25/B25)</x:f>
-        <x:v>1.15</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="H25" s="25" t="n">
         <x:f>IF(OR(B25=0,D25=""),"",MAX(B25-D25,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I25" s="27" t="str">
-        <x:f>IF(B25=0,"Sin meta",IF(D25="","Sin dato financiero",IF(D25&gt;B25,"Superada",IF(D25=B25,"Cumplida",IF(G25&gt;=0.8,"Cerca",IF(G25&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B25=0,"Sin meta",IF(D25="","Sin dato financiero",IF(D25&gt;B25,"Superada",IF(D25=B25,"Cumplida",IF(D25/B25&gt;=0.8,"Cerca",IF(D25/B25&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J25" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1434,10 +1433,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D26" s="25" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E26" s="25" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F26" s="25" t="n">
         <x:f>IF(D26="","",E26-D26)</x:f>
@@ -1445,18 +1444,18 @@
       </x:c>
       <x:c r="G26" s="26" t="n">
         <x:f>IF(OR(B26=0,D26=""),"",D26/B26)</x:f>
-        <x:v>0.7</x:v>
+        <x:v>0.725</x:v>
       </x:c>
       <x:c r="H26" s="25" t="n">
         <x:f>IF(OR(B26=0,D26=""),"",MAX(B26-D26,0))</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="I26" s="27" t="str">
-        <x:f>IF(B26=0,"Sin meta",IF(D26="","Sin dato financiero",IF(D26&gt;B26,"Superada",IF(D26=B26,"Cumplida",IF(G26&gt;=0.8,"Cerca",IF(G26&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B26=0,"Sin meta",IF(D26="","Sin dato financiero",IF(D26&gt;B26,"Superada",IF(D26=B26,"Cumplida",IF(D26/B26&gt;=0.8,"Cerca",IF(D26/B26&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J26" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1471,10 +1470,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D27" s="25" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E27" s="25" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F27" s="25" t="n">
         <x:f>IF(D27="","",E27-D27)</x:f>
@@ -1482,18 +1481,18 @@
       </x:c>
       <x:c r="G27" s="26" t="n">
         <x:f>IF(OR(B27=0,D27=""),"",D27/B27)</x:f>
-        <x:v>1</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="H27" s="25" t="n">
         <x:f>IF(OR(B27=0,D27=""),"",MAX(B27-D27,0))</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I27" s="27" t="str">
-        <x:f>IF(B27=0,"Sin meta",IF(D27="","Sin dato financiero",IF(D27&gt;B27,"Superada",IF(D27=B27,"Cumplida",IF(G27&gt;=0.8,"Cerca",IF(G27&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
-        <x:v>Cumplida</x:v>
+        <x:f>IF(B27=0,"Sin meta",IF(D27="","Sin dato financiero",IF(D27&gt;B27,"Superada",IF(D27=B27,"Cumplida",IF(D27/B27&gt;=0.8,"Cerca",IF(D27/B27&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:v>Superada</x:v>
       </x:c>
       <x:c r="J27" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1526,11 +1525,11 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="I28" s="27" t="str">
-        <x:f>IF(B28=0,"Sin meta",IF(D28="","Sin dato financiero",IF(D28&gt;B28,"Superada",IF(D28=B28,"Cumplida",IF(G28&gt;=0.8,"Cerca",IF(G28&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B28=0,"Sin meta",IF(D28="","Sin dato financiero",IF(D28&gt;B28,"Superada",IF(D28=B28,"Cumplida",IF(D28/B28&gt;=0.8,"Cerca",IF(D28/B28&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Cerca</x:v>
       </x:c>
       <x:c r="J28" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1558,11 +1557,11 @@
         <x:f>IF(OR(B29=0,D29=""),"",MAX(B29-D29,0))</x:f>
       </x:c>
       <x:c r="I29" s="27" t="str">
-        <x:f>IF(B29=0,"Sin meta",IF(D29="","Sin dato financiero",IF(D29&gt;B29,"Superada",IF(D29=B29,"Cumplida",IF(G29&gt;=0.8,"Cerca",IF(G29&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B29=0,"Sin meta",IF(D29="","Sin dato financiero",IF(D29&gt;B29,"Superada",IF(D29=B29,"Cumplida",IF(D29/B29&gt;=0.8,"Cerca",IF(D29/B29&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Sin dato financiero</x:v>
       </x:c>
       <x:c r="J29" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1595,11 +1594,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I30" s="27" t="str">
-        <x:f>IF(B30=0,"Sin meta",IF(D30="","Sin dato financiero",IF(D30&gt;B30,"Superada",IF(D30=B30,"Cumplida",IF(G30&gt;=0.8,"Cerca",IF(G30&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B30=0,"Sin meta",IF(D30="","Sin dato financiero",IF(D30&gt;B30,"Superada",IF(D30=B30,"Cumplida",IF(D30/B30&gt;=0.8,"Cerca",IF(D30/B30&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J30" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1632,11 +1631,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I31" s="32" t="str">
-        <x:f>IF(B31=0,"Sin meta",IF(D31="","Sin dato financiero",IF(D31&gt;B31,"Superada",IF(D31=B31,"Cumplida",IF(G31&gt;=0.8,"Cerca",IF(G31&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
+        <x:f>IF(B31=0,"Sin meta",IF(D31="","Sin dato financiero",IF(D31&gt;B31,"Superada",IF(D31=B31,"Cumplida",IF(D31/B31&gt;=0.8,"Cerca",IF(D31/B31&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J31" s="33" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 12-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1666,7 +1665,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Nivel 1 del reporte institucional matr83 · 12 de agosto de 2026, 15:37</x:v>
+        <x:v>Nivel 1 del reporte institucional MATR83 · 18 de agosto de 2026, 14:58</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1720,7 +1719,7 @@
         <x:v>Administración de Servicios de Salud</x:v>
       </x:c>
       <x:c r="B8" s="19" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1731,7 +1730,7 @@
         <x:v>Arquitectura</x:v>
       </x:c>
       <x:c r="B9" s="19" t="n">
-        <x:v>29</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1753,7 +1752,7 @@
         <x:v>Comunicación Social y Medios Digitales</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C11" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1764,7 +1763,7 @@
         <x:v>Contaduría Pública</x:v>
       </x:c>
       <x:c r="B12" s="19" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1775,7 +1774,7 @@
         <x:v>Creación y Diseño</x:v>
       </x:c>
       <x:c r="B13" s="19" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1786,7 +1785,7 @@
         <x:v>Derecho</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C14" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1797,7 +1796,7 @@
         <x:v>Derecho Villavicencio</x:v>
       </x:c>
       <x:c r="B15" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C15" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1819,7 +1818,7 @@
         <x:v>Ingeniería Civil</x:v>
       </x:c>
       <x:c r="B17" s="19" t="n">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C17" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1830,7 +1829,7 @@
         <x:v>Ingeniería de Sistemas</x:v>
       </x:c>
       <x:c r="B18" s="19" t="n">
-        <x:v>48</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C18" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1841,7 +1840,7 @@
         <x:v>Ingeniería Eléctrica</x:v>
       </x:c>
       <x:c r="B19" s="19" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C19" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1874,7 +1873,7 @@
         <x:v>Ingeniería Mecánica</x:v>
       </x:c>
       <x:c r="B22" s="19" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C22" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1896,7 +1895,7 @@
         <x:v>Mercadeo y Publicidad</x:v>
       </x:c>
       <x:c r="B24" s="19" t="n">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C24" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1907,7 +1906,7 @@
         <x:v>Negocios Internacionales</x:v>
       </x:c>
       <x:c r="B25" s="19" t="n">
-        <x:v>51</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C25" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1918,7 +1917,7 @@
         <x:v>Psicología</x:v>
       </x:c>
       <x:c r="B26" s="19" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C26" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1929,7 +1928,7 @@
         <x:v>Psicología Villavicencio</x:v>
       </x:c>
       <x:c r="B27" s="19" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -2014,7 +2013,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Inscripción normal + reserva de cupo · Barranquilla y Villavicencio · 12 de agosto de 2026</x:v>
+        <x:v>Inscripción normal + reserva de cupo · Barranquilla y Villavicencio · 18 de agosto de 2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2063,11 +2062,11 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="20" t="n">
-        <x:f>E5/B5</x:f>
+        <x:f>IF(B5=0,"",E5/B5)</x:f>
         <x:v>0.1984126984126984</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2081,17 +2080,17 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="D6" s="19" t="n">
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E6" s="19" t="n">
-        <x:v>34</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F6" s="20" t="n">
-        <x:f>E6/B6</x:f>
-        <x:v>0.4657534246575342</x:v>
+        <x:f>IF(B6=0,"",E6/B6)</x:f>
+        <x:v>0.4931506849315068</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2111,11 +2110,11 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="F7" s="20" t="n">
-        <x:f>E7/B7</x:f>
+        <x:f>IF(B7=0,"",E7/B7)</x:f>
         <x:v>0.4583333333333333</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2132,14 +2131,14 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E8" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F8" s="20" t="n">
-        <x:f>E8/B8</x:f>
-        <x:v>0.3333333333333333</x:v>
+        <x:f>IF(B8=0,"",E8/B8)</x:f>
+        <x:v>0.375</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2159,11 +2158,11 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="F9" s="20" t="n">
-        <x:f>E9/B9</x:f>
+        <x:f>IF(B9=0,"",E9/B9)</x:f>
         <x:v>0.6923076923076923</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2183,11 +2182,11 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="F10" s="20" t="n">
-        <x:f>E10/B10</x:f>
+        <x:f>IF(B10=0,"",E10/B10)</x:f>
         <x:v>0.4915254237288136</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2204,14 +2203,14 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="E11" s="19" t="n">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F11" s="20" t="n">
-        <x:f>E11/B11</x:f>
-        <x:v>0.45569620253164556</x:v>
+        <x:f>IF(B11=0,"",E11/B11)</x:f>
+        <x:v>0.4936708860759494</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2231,11 +2230,11 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F12" s="20" t="n">
-        <x:f>E12/B12</x:f>
+        <x:f>IF(B12=0,"",E12/B12)</x:f>
         <x:v>0.42857142857142855</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2246,20 +2245,20 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="C13" s="19" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D13" s="19" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="E13" s="19" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F13" s="20" t="n">
-        <x:f>E13/B13</x:f>
-        <x:v>0.4222222222222222</x:v>
+        <x:f>IF(B13=0,"",E13/B13)</x:f>
+        <x:v>0.4444444444444444</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2267,23 +2266,23 @@
         <x:v>Creación y Diseño</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C14" s="19" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D14" s="19" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E14" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F14" s="20" t="n">
-        <x:f>E14/B14</x:f>
-        <x:v>0.47058823529411764</x:v>
+        <x:f>IF(B14=0,"",E14/B14)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2300,14 +2299,14 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="E15" s="19" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F15" s="20" t="n">
-        <x:f>E15/B15</x:f>
-        <x:v>0.36363636363636365</x:v>
+        <x:f>IF(B15=0,"",E15/B15)</x:f>
+        <x:v>0.38636363636363635</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2324,14 +2323,14 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E16" s="19" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F16" s="20" t="n">
-        <x:f>E16/B16</x:f>
-        <x:v>0.5833333333333334</x:v>
+        <x:f>IF(B16=0,"",E16/B16)</x:f>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2339,10 +2338,10 @@
         <x:v>Técnico en Desarrollo de Software</x:v>
       </x:c>
       <x:c r="B17" s="19" t="n">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C17" s="19" t="n">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D17" s="19" t="n">
         <x:v>42</x:v>
@@ -2351,11 +2350,11 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="F17" s="20" t="n">
-        <x:f>E17/B17</x:f>
-        <x:v>0.5964912280701754</x:v>
+        <x:f>IF(B17=0,"",E17/B17)</x:f>
+        <x:v>0.5862068965517241</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2363,7 +2362,7 @@
         <x:v>Administración de Empresas</x:v>
       </x:c>
       <x:c r="B18" s="19" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C18" s="19" t="n">
         <x:v>47</x:v>
@@ -2375,11 +2374,11 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F18" s="20" t="n">
-        <x:f>E18/B18</x:f>
-        <x:v>0.546875</x:v>
+        <x:f>IF(B18=0,"",E18/B18)</x:f>
+        <x:v>0.5384615384615384</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2387,7 +2386,7 @@
         <x:v>Contaduría Pública</x:v>
       </x:c>
       <x:c r="B19" s="19" t="n">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C19" s="19" t="n">
         <x:v>35</x:v>
@@ -2396,14 +2395,14 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="E19" s="19" t="n">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F19" s="20" t="n">
-        <x:f>E19/B19</x:f>
-        <x:v>0.5576923076923077</x:v>
+        <x:f>IF(B19=0,"",E19/B19)</x:f>
+        <x:v>0.5660377358490566</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2411,23 +2410,23 @@
         <x:v>Negocios Internacionales</x:v>
       </x:c>
       <x:c r="B20" s="19" t="n">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C20" s="19" t="n">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D20" s="19" t="n">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E20" s="19" t="n">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="F20" s="20" t="n">
-        <x:f>E20/B20</x:f>
-        <x:v>0.5476190476190477</x:v>
+        <x:f>IF(B20=0,"",E20/B20)</x:f>
+        <x:v>0.5647058823529412</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2438,7 +2437,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="C21" s="19" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D21" s="19" t="n">
         <x:v>14</x:v>
@@ -2447,11 +2446,11 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="F21" s="20" t="n">
-        <x:f>E21/B21</x:f>
+        <x:f>IF(B21=0,"",E21/B21)</x:f>
         <x:v>0.56</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2468,14 +2467,14 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="E22" s="19" t="n">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F22" s="20" t="n">
-        <x:f>E22/B22</x:f>
-        <x:v>0.7142857142857143</x:v>
+        <x:f>IF(B22=0,"",E22/B22)</x:f>
+        <x:v>0.7346938775510204</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2492,14 +2491,14 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="E23" s="19" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F23" s="20" t="n">
-        <x:f>E23/B23</x:f>
-        <x:v>0.4827586206896552</x:v>
+        <x:f>IF(B23=0,"",E23/B23)</x:f>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2516,14 +2515,14 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E24" s="19" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="20" t="n">
-        <x:f>E24/B24</x:f>
-        <x:v>0.5</x:v>
+        <x:f>IF(B24=0,"",E24/B24)</x:f>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2531,23 +2530,23 @@
         <x:v>Comunicación Social y Medios Digitales</x:v>
       </x:c>
       <x:c r="B25" s="19" t="n">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C25" s="19" t="n">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D25" s="19" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="E25" s="19" t="n">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F25" s="20" t="n">
-        <x:f>E25/B25</x:f>
-        <x:v>0.6216216216216216</x:v>
+        <x:f>IF(B25=0,"",E25/B25)</x:f>
+        <x:v>0.6578947368421053</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2567,11 +2566,11 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F26" s="20" t="n">
-        <x:f>E26/B26</x:f>
+        <x:f>IF(B26=0,"",E26/B26)</x:f>
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>EINR41 PS + RC · 12-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Actualiza matriculas al corte del 19 de agosto
</commit_message>
<xml_diff>
--- a/Dashboard_Matriculas_CUC_2026-2.xlsx
+++ b/Dashboard_Matriculas_CUC_2026-2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen ejecutivo" sheetId="1" r:id="R7863787f1a794e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado por programa" sheetId="2" r:id="R9e678147996749c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrícula académica" sheetId="3" r:id="Ra09e180092844861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embudo de admisiones" sheetId="4" r:id="R9749fc450c424dc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen ejecutivo" sheetId="1" r:id="R38995d6ea4004e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado por programa" sheetId="2" r:id="R956ef478eb8e4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrícula académica" sheetId="3" r:id="R3c59269d48944e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embudo de admisiones" sheetId="4" r:id="R675b7f29de424706"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -459,7 +459,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Corte institucional del 18 de agosto de 2026 · Cumplimiento basado en matrícula financiera</x:v>
+        <x:v>Corte institucional del 19 de agosto de 2026 · Cumplimiento basado en matrícula financiera</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -494,7 +494,7 @@
       </x:c>
       <x:c r="E5" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!B5:B26)</x:f>
-        <x:v>991</x:v>
+        <x:v>996</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -503,14 +503,14 @@
       </x:c>
       <x:c r="B6" s="13" t="n">
         <x:f>SUM('Consolidado por programa'!D5:D31)</x:f>
-        <x:v>487</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
         <x:v>Inscritos</x:v>
       </x:c>
       <x:c r="E6" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!C5:C26)</x:f>
-        <x:v>672</x:v>
+        <x:v>676</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -519,14 +519,14 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>IF(B5=0,0,B6/B5)</x:f>
-        <x:v>0.8650088809946714</x:v>
+        <x:v>0.8632326820603907</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
         <x:v>Admitidos</x:v>
       </x:c>
       <x:c r="E7" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!D5:D26)</x:f>
-        <x:v>624</x:v>
+        <x:v>625</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -535,14 +535,14 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>MAX(B5-B6,0)</x:f>
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
         <x:v>Por admitir</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
         <x:f>MAX(E5-E7-E9,0)</x:f>
-        <x:v>366</x:v>
+        <x:v>370</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -551,7 +551,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>SUM('Consolidado por programa'!E5:E31)</x:f>
-        <x:v>568</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Rechazados</x:v>
@@ -562,7 +562,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18" t="str">
-        <x:v>Lectura: 487 estudiantes han completado la matrícula financiera. Las 568 matrículas académicas de primer nivel representan 81 estudiantes de diferencia respecto al pago y funcionan como indicador complementario de proximidad.</x:v>
+        <x:v>Lectura: 486 estudiantes han completado la matrícula financiera. Las 571 matrículas académicas de primer nivel representan 85 estudiantes de diferencia respecto al pago y funcionan como indicador complementario de proximidad.</x:v>
       </x:c>
       <x:c r="B11" s="18"/>
       <x:c r="C11" s="18"/>
@@ -620,7 +620,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Metas, matrícula financiera y matrícula académica · Periodo 2026-2 · Corte 18 de agosto de 2026</x:v>
+        <x:v>Metas, matrícula financiera y matrícula académica · Periodo 2026-2 · Corte 19 de agosto de 2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -693,7 +693,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J5" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -730,7 +730,7 @@
         <x:v>Cumplida</x:v>
       </x:c>
       <x:c r="J6" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -762,7 +762,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J7" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -777,10 +777,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D8" s="25" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E8" s="25" t="n">
         <x:v>14</x:v>
-      </x:c>
-      <x:c r="E8" s="25" t="n">
-        <x:v>15</x:v>
       </x:c>
       <x:c r="F8" s="25" t="n">
         <x:f>IF(D8="","",E8-D8)</x:f>
@@ -788,7 +788,7 @@
       </x:c>
       <x:c r="G8" s="26" t="n">
         <x:f>IF(OR(B8=0,D8=""),"",D8/B8)</x:f>
-        <x:v>1.75</x:v>
+        <x:v>1.625</x:v>
       </x:c>
       <x:c r="H8" s="25" t="n">
         <x:f>IF(OR(B8=0,D8=""),"",MAX(B8-D8,0))</x:f>
@@ -799,7 +799,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J8" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -836,7 +836,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J9" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -868,7 +868,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J10" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -905,7 +905,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J11" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -920,10 +920,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D12" s="25" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E12" s="25" t="n">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F12" s="25" t="n">
         <x:f>IF(D12="","",E12-D12)</x:f>
@@ -931,7 +931,7 @@
       </x:c>
       <x:c r="G12" s="26" t="n">
         <x:f>IF(OR(B12=0,D12=""),"",D12/B12)</x:f>
-        <x:v>1.3636363636363635</x:v>
+        <x:v>1.3181818181818181</x:v>
       </x:c>
       <x:c r="H12" s="25" t="n">
         <x:f>IF(OR(B12=0,D12=""),"",MAX(B12-D12,0))</x:f>
@@ -942,7 +942,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J12" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -979,7 +979,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J13" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -997,11 +997,11 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="E14" s="25" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F14" s="25" t="n">
         <x:f>IF(D14="","",E14-D14)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G14" s="26" t="n">
         <x:f>IF(OR(B14=0,D14=""),"",D14/B14)</x:f>
@@ -1016,7 +1016,7 @@
         <x:v>Rezagada</x:v>
       </x:c>
       <x:c r="J14" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1053,7 +1053,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J15" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1090,7 +1090,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J16" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1105,10 +1105,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D17" s="25" t="n">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E17" s="25" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F17" s="25" t="n">
         <x:f>IF(D17="","",E17-D17)</x:f>
@@ -1116,18 +1116,18 @@
       </x:c>
       <x:c r="G17" s="26" t="n">
         <x:f>IF(OR(B17=0,D17=""),"",D17/B17)</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.7708333333333334</x:v>
       </x:c>
       <x:c r="H17" s="25" t="n">
         <x:f>IF(OR(B17=0,D17=""),"",MAX(B17-D17,0))</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="I17" s="27" t="str">
         <x:f>IF(B17=0,"Sin meta",IF(D17="","Sin dato financiero",IF(D17&gt;B17,"Superada",IF(D17=B17,"Cumplida",IF(D17/B17&gt;=0.8,"Cerca",IF(D17/B17&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J17" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1145,11 +1145,11 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="E18" s="25" t="n">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F18" s="25" t="n">
         <x:f>IF(D18="","",E18-D18)</x:f>
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G18" s="26" t="n">
         <x:f>IF(OR(B18=0,D18=""),"",D18/B18)</x:f>
@@ -1164,7 +1164,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J18" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1182,11 +1182,11 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E19" s="25" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F19" s="25" t="n">
         <x:f>IF(D19="","",E19-D19)</x:f>
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G19" s="26" t="n">
         <x:f>IF(OR(B19=0,D19=""),"",D19/B19)</x:f>
@@ -1201,7 +1201,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J19" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1219,11 +1219,11 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E20" s="25" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F20" s="25" t="n">
         <x:f>IF(D20="","",E20-D20)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G20" s="26" t="n">
         <x:f>IF(OR(B20=0,D20=""),"",D20/B20)</x:f>
@@ -1238,7 +1238,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J20" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1253,10 +1253,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D21" s="25" t="n">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E21" s="25" t="n">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F21" s="25" t="n">
         <x:f>IF(D21="","",E21-D21)</x:f>
@@ -1264,18 +1264,18 @@
       </x:c>
       <x:c r="G21" s="26" t="n">
         <x:f>IF(OR(B21=0,D21=""),"",D21/B21)</x:f>
-        <x:v>0.9666666666666667</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H21" s="25" t="n">
         <x:f>IF(OR(B21=0,D21=""),"",MAX(B21-D21,0))</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I21" s="27" t="str">
         <x:f>IF(B21=0,"Sin meta",IF(D21="","Sin dato financiero",IF(D21&gt;B21,"Superada",IF(D21=B21,"Cumplida",IF(D21/B21&gt;=0.8,"Cerca",IF(D21/B21&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
-        <x:v>Cerca</x:v>
+        <x:v>Cumplida</x:v>
       </x:c>
       <x:c r="J21" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1312,7 +1312,7 @@
         <x:v>Rezagada</x:v>
       </x:c>
       <x:c r="J22" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1344,7 +1344,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J23" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1381,7 +1381,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J24" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1418,7 +1418,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J25" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1455,7 +1455,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J26" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1492,7 +1492,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J27" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1529,7 +1529,7 @@
         <x:v>Cerca</x:v>
       </x:c>
       <x:c r="J28" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1561,7 +1561,7 @@
         <x:v>Sin dato financiero</x:v>
       </x:c>
       <x:c r="J29" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1576,10 +1576,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D30" s="25" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E30" s="25" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F30" s="25" t="n">
         <x:f>IF(D30="","",E30-D30)</x:f>
@@ -1587,7 +1587,7 @@
       </x:c>
       <x:c r="G30" s="26" t="n">
         <x:f>IF(OR(B30=0,D30=""),"",D30/B30)</x:f>
-        <x:v>1.5</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="H30" s="25" t="n">
         <x:f>IF(OR(B30=0,D30=""),"",MAX(B30-D30,0))</x:f>
@@ -1598,7 +1598,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J30" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1635,7 +1635,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J31" s="33" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 18-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1665,7 +1665,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Nivel 1 del reporte institucional MATR83 · 18 de agosto de 2026, 14:58</x:v>
+        <x:v>Nivel 1 del reporte institucional MATR83 · 19 de agosto de 2026, 15:18</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1719,7 +1719,7 @@
         <x:v>Administración de Servicios de Salud</x:v>
       </x:c>
       <x:c r="B8" s="19" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1763,7 +1763,7 @@
         <x:v>Contaduría Pública</x:v>
       </x:c>
       <x:c r="B12" s="19" t="n">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1785,7 +1785,7 @@
         <x:v>Derecho</x:v>
       </x:c>
       <x:c r="B14" s="19" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C14" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1818,7 +1818,7 @@
         <x:v>Ingeniería Civil</x:v>
       </x:c>
       <x:c r="B17" s="19" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C17" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1829,7 +1829,7 @@
         <x:v>Ingeniería de Sistemas</x:v>
       </x:c>
       <x:c r="B18" s="19" t="n">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C18" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1840,7 +1840,7 @@
         <x:v>Ingeniería Eléctrica</x:v>
       </x:c>
       <x:c r="B19" s="19" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C19" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1851,7 +1851,7 @@
         <x:v>Ingeniería Electrónica</x:v>
       </x:c>
       <x:c r="B20" s="19" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C20" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1862,7 +1862,7 @@
         <x:v>Ingeniería Industrial</x:v>
       </x:c>
       <x:c r="B21" s="19" t="n">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C21" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1961,7 +1961,7 @@
         <x:v>Técnico en Entrenamiento Deportivo</x:v>
       </x:c>
       <x:c r="B30" s="19" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C30" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -2013,7 +2013,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Inscripción normal + reserva de cupo · Barranquilla y Villavicencio · 18 de agosto de 2026</x:v>
+        <x:v>Inscripción normal + reserva de cupo · Barranquilla y Villavicencio · 19 de agosto de 2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2066,7 +2066,7 @@
         <x:v>0.1984126984126984</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2074,23 +2074,23 @@
         <x:v>Ingeniería Civil</x:v>
       </x:c>
       <x:c r="B6" s="19" t="n">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C6" s="19" t="n">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D6" s="19" t="n">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E6" s="19" t="n">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F6" s="20" t="n">
         <x:f>IF(B6=0,"",E6/B6)</x:f>
-        <x:v>0.4931506849315068</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2114,7 +2114,7 @@
         <x:v>0.4583333333333333</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2138,7 +2138,7 @@
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2162,7 +2162,7 @@
         <x:v>0.6923076923076923</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2179,14 +2179,14 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="E10" s="19" t="n">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F10" s="20" t="n">
         <x:f>IF(B10=0,"",E10/B10)</x:f>
-        <x:v>0.4915254237288136</x:v>
+        <x:v>0.5084745762711864</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2210,7 +2210,7 @@
         <x:v>0.4936708860759494</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2234,7 +2234,7 @@
         <x:v>0.42857142857142855</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2258,7 +2258,7 @@
         <x:v>0.4444444444444444</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2269,7 +2269,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="C14" s="19" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D14" s="19" t="n">
         <x:v>12</x:v>
@@ -2282,7 +2282,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2306,7 +2306,7 @@
         <x:v>0.38636363636363635</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2330,7 +2330,7 @@
         <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2338,10 +2338,10 @@
         <x:v>Técnico en Desarrollo de Software</x:v>
       </x:c>
       <x:c r="B17" s="19" t="n">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C17" s="19" t="n">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D17" s="19" t="n">
         <x:v>42</x:v>
@@ -2351,10 +2351,10 @@
       </x:c>
       <x:c r="F17" s="20" t="n">
         <x:f>IF(B17=0,"",E17/B17)</x:f>
-        <x:v>0.5862068965517241</x:v>
+        <x:v>0.576271186440678</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2362,7 +2362,7 @@
         <x:v>Administración de Empresas</x:v>
       </x:c>
       <x:c r="B18" s="19" t="n">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C18" s="19" t="n">
         <x:v>47</x:v>
@@ -2375,10 +2375,10 @@
       </x:c>
       <x:c r="F18" s="20" t="n">
         <x:f>IF(B18=0,"",E18/B18)</x:f>
-        <x:v>0.5384615384615384</x:v>
+        <x:v>0.5303030303030303</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2389,20 +2389,20 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="C19" s="19" t="n">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D19" s="19" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="E19" s="19" t="n">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F19" s="20" t="n">
         <x:f>IF(B19=0,"",E19/B19)</x:f>
-        <x:v>0.5660377358490566</x:v>
+        <x:v>0.5471698113207547</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2426,7 +2426,7 @@
         <x:v>0.5647058823529412</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2443,14 +2443,14 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E21" s="19" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F21" s="20" t="n">
         <x:f>IF(B21=0,"",E21/B21)</x:f>
-        <x:v>0.56</x:v>
+        <x:v>0.52</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2474,7 +2474,7 @@
         <x:v>0.7346938775510204</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2498,7 +2498,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2522,7 +2522,7 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2530,7 +2530,7 @@
         <x:v>Comunicación Social y Medios Digitales</x:v>
       </x:c>
       <x:c r="B25" s="19" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C25" s="19" t="n">
         <x:v>32</x:v>
@@ -2543,10 +2543,10 @@
       </x:c>
       <x:c r="F25" s="20" t="n">
         <x:f>IF(B25=0,"",E25/B25)</x:f>
-        <x:v>0.6578947368421053</x:v>
+        <x:v>0.6410256410256411</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2554,7 +2554,7 @@
         <x:v>Técnico en Entrenamiento Deportivo</x:v>
       </x:c>
       <x:c r="B26" s="19" t="n">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C26" s="19" t="n">
         <x:v>18</x:v>
@@ -2563,14 +2563,14 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E26" s="19" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F26" s="20" t="n">
         <x:f>IF(B26=0,"",E26/B26)</x:f>
-        <x:v>0.6</x:v>
+        <x:v>0.5384615384615384</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>EINR41 PS + RC · 18-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Actualizar dashboard al corte del 21 de agosto de 2026
</commit_message>
<xml_diff>
--- a/Dashboard_Matriculas_CUC_2026-2.xlsx
+++ b/Dashboard_Matriculas_CUC_2026-2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen ejecutivo" sheetId="1" r:id="R38995d6ea4004e94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado por programa" sheetId="2" r:id="R956ef478eb8e4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrícula académica" sheetId="3" r:id="R3c59269d48944e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embudo de admisiones" sheetId="4" r:id="R675b7f29de424706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen ejecutivo" sheetId="1" r:id="R28178ac632d84478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidado por programa" sheetId="2" r:id="R6757c566d45242f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrícula académica" sheetId="3" r:id="R64e12b4a754240cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Embudo de admisiones" sheetId="4" r:id="R43e421676a2c4e6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -459,7 +459,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Corte institucional del 19 de agosto de 2026 · Cumplimiento basado en matrícula financiera</x:v>
+        <x:v>Corte institucional del 21 de agosto de 2026 · Cumplimiento basado en matrícula financiera</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -494,7 +494,7 @@
       </x:c>
       <x:c r="E5" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!B5:B26)</x:f>
-        <x:v>996</x:v>
+        <x:v>997</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -503,14 +503,14 @@
       </x:c>
       <x:c r="B6" s="13" t="n">
         <x:f>SUM('Consolidado por programa'!D5:D31)</x:f>
-        <x:v>486</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
         <x:v>Inscritos</x:v>
       </x:c>
       <x:c r="E6" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!C5:C26)</x:f>
-        <x:v>676</x:v>
+        <x:v>678</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -519,14 +519,14 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>IF(B5=0,0,B6/B5)</x:f>
-        <x:v>0.8632326820603907</x:v>
+        <x:v>0.8650088809946714</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
         <x:v>Admitidos</x:v>
       </x:c>
       <x:c r="E7" s="13" t="n">
         <x:f>SUM('Embudo de admisiones'!D5:D26)</x:f>
-        <x:v>625</x:v>
+        <x:v>628</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -535,14 +535,14 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>MAX(B5-B6,0)</x:f>
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
         <x:v>Por admitir</x:v>
       </x:c>
       <x:c r="E8" s="13" t="n">
         <x:f>MAX(E5-E7-E9,0)</x:f>
-        <x:v>370</x:v>
+        <x:v>368</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -551,7 +551,7 @@
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:f>SUM('Consolidado por programa'!E5:E31)</x:f>
-        <x:v>571</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
         <x:v>Rechazados</x:v>
@@ -562,7 +562,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18" t="str">
-        <x:v>Lectura: 486 estudiantes han completado la matrícula financiera. Las 571 matrículas académicas de primer nivel representan 85 estudiantes de diferencia respecto al pago y funcionan como indicador complementario de proximidad.</x:v>
+        <x:v>Lectura: 487 estudiantes han completado la matrícula financiera. Las 572 matrículas académicas de primer nivel representan 85 estudiantes de diferencia respecto al pago y funcionan como indicador complementario de proximidad.</x:v>
       </x:c>
       <x:c r="B11" s="18"/>
       <x:c r="C11" s="18"/>
@@ -620,7 +620,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Metas, matrícula financiera y matrícula académica · Periodo 2026-2 · Corte 19 de agosto de 2026</x:v>
+        <x:v>Metas, matrícula financiera y matrícula académica · Periodo 2026-2 · Corte 21 de agosto de 2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -693,7 +693,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J5" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -730,7 +730,7 @@
         <x:v>Cumplida</x:v>
       </x:c>
       <x:c r="J6" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -762,7 +762,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J7" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -799,7 +799,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J8" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -814,29 +814,29 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D9" s="25" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E9" s="25" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F9" s="25" t="n">
         <x:f>IF(D9="","",E9-D9)</x:f>
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G9" s="26" t="n">
         <x:f>IF(OR(B9=0,D9=""),"",D9/B9)</x:f>
-        <x:v>0.5555555555555556</x:v>
+        <x:v>0.5277777777777778</x:v>
       </x:c>
       <x:c r="H9" s="25" t="n">
         <x:f>IF(OR(B9=0,D9=""),"",MAX(B9-D9,0))</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I9" s="27" t="str">
         <x:f>IF(B9=0,"Sin meta",IF(D9="","Sin dato financiero",IF(D9&gt;B9,"Superada",IF(D9=B9,"Cumplida",IF(D9/B9&gt;=0.8,"Cerca",IF(D9/B9&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J9" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -868,7 +868,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J10" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -905,7 +905,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J11" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -942,7 +942,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J12" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -979,7 +979,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J13" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1016,7 +1016,7 @@
         <x:v>Rezagada</x:v>
       </x:c>
       <x:c r="J14" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1053,7 +1053,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J15" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1090,7 +1090,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J16" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1105,29 +1105,29 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D17" s="25" t="n">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E17" s="25" t="n">
         <x:v>44</x:v>
       </x:c>
       <x:c r="F17" s="25" t="n">
         <x:f>IF(D17="","",E17-D17)</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G17" s="26" t="n">
         <x:f>IF(OR(B17=0,D17=""),"",D17/B17)</x:f>
-        <x:v>0.7708333333333334</x:v>
+        <x:v>0.7916666666666666</x:v>
       </x:c>
       <x:c r="H17" s="25" t="n">
         <x:f>IF(OR(B17=0,D17=""),"",MAX(B17-D17,0))</x:f>
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="I17" s="27" t="str">
         <x:f>IF(B17=0,"Sin meta",IF(D17="","Sin dato financiero",IF(D17&gt;B17,"Superada",IF(D17=B17,"Cumplida",IF(D17/B17&gt;=0.8,"Cerca",IF(D17/B17&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J17" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1164,7 +1164,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J18" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1182,11 +1182,11 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E19" s="25" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F19" s="25" t="n">
         <x:f>IF(D19="","",E19-D19)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G19" s="26" t="n">
         <x:f>IF(OR(B19=0,D19=""),"",D19/B19)</x:f>
@@ -1201,7 +1201,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J19" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1238,7 +1238,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J20" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1256,11 +1256,11 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="E21" s="25" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F21" s="25" t="n">
         <x:f>IF(D21="","",E21-D21)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G21" s="26" t="n">
         <x:f>IF(OR(B21=0,D21=""),"",D21/B21)</x:f>
@@ -1275,7 +1275,7 @@
         <x:v>Cumplida</x:v>
       </x:c>
       <x:c r="J21" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1312,7 +1312,7 @@
         <x:v>Rezagada</x:v>
       </x:c>
       <x:c r="J22" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1344,7 +1344,7 @@
         <x:v>Sin meta</x:v>
       </x:c>
       <x:c r="J23" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1381,7 +1381,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J24" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1399,11 +1399,11 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E25" s="25" t="n">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F25" s="25" t="n">
         <x:f>IF(D25="","",E25-D25)</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G25" s="26" t="n">
         <x:f>IF(OR(B25=0,D25=""),"",D25/B25)</x:f>
@@ -1418,7 +1418,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J25" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1455,7 +1455,7 @@
         <x:v>En progreso</x:v>
       </x:c>
       <x:c r="J26" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1492,7 +1492,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J27" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1507,10 +1507,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D28" s="25" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E28" s="25" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F28" s="25" t="n">
         <x:f>IF(D28="","",E28-D28)</x:f>
@@ -1518,18 +1518,18 @@
       </x:c>
       <x:c r="G28" s="26" t="n">
         <x:f>IF(OR(B28=0,D28=""),"",D28/B28)</x:f>
-        <x:v>0.85</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="H28" s="25" t="n">
         <x:f>IF(OR(B28=0,D28=""),"",MAX(B28-D28,0))</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I28" s="27" t="str">
         <x:f>IF(B28=0,"Sin meta",IF(D28="","Sin dato financiero",IF(D28&gt;B28,"Superada",IF(D28=B28,"Cumplida",IF(D28/B28&gt;=0.8,"Cerca",IF(D28/B28&gt;=0.5,"En progreso","Rezagada"))))))</x:f>
         <x:v>Cerca</x:v>
       </x:c>
       <x:c r="J28" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1561,7 +1561,7 @@
         <x:v>Sin dato financiero</x:v>
       </x:c>
       <x:c r="J29" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1598,7 +1598,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J30" s="28" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1635,7 +1635,7 @@
         <x:v>Superada</x:v>
       </x:c>
       <x:c r="J31" s="33" t="str">
-        <x:v>MATR83 + EINR41 PS/RC · 19-08-2026</x:v>
+        <x:v>MATR83 + EINR41 PS/RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1665,7 +1665,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Nivel 1 del reporte institucional MATR83 · 19 de agosto de 2026, 15:18</x:v>
+        <x:v>Nivel 1 del reporte institucional MATR83 · 21 de agosto de 2026, 15:09</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1730,7 +1730,7 @@
         <x:v>Arquitectura</x:v>
       </x:c>
       <x:c r="B9" s="19" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1840,7 +1840,7 @@
         <x:v>Ingeniería Eléctrica</x:v>
       </x:c>
       <x:c r="B19" s="19" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C19" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1862,7 +1862,7 @@
         <x:v>Ingeniería Industrial</x:v>
       </x:c>
       <x:c r="B21" s="19" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C21" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1906,7 +1906,7 @@
         <x:v>Negocios Internacionales</x:v>
       </x:c>
       <x:c r="B25" s="19" t="n">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C25" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -1939,7 +1939,7 @@
         <x:v>Técnico en Desarrollo de Software</x:v>
       </x:c>
       <x:c r="B28" s="19" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C28" t="str">
         <x:v>Primer nivel / semestre</x:v>
@@ -2013,7 +2013,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Inscripción normal + reserva de cupo · Barranquilla y Villavicencio · 19 de agosto de 2026</x:v>
+        <x:v>Inscripción normal + reserva de cupo · Barranquilla y Villavicencio · 21 de agosto de 2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2066,7 +2066,7 @@
         <x:v>0.1984126984126984</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2080,17 +2080,17 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="D6" s="19" t="n">
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E6" s="19" t="n">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F6" s="20" t="n">
         <x:f>IF(B6=0,"",E6/B6)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.5135135135135135</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2114,7 +2114,7 @@
         <x:v>0.4583333333333333</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2138,7 +2138,7 @@
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2162,7 +2162,7 @@
         <x:v>0.6923076923076923</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2186,7 +2186,7 @@
         <x:v>0.5084745762711864</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2210,7 +2210,7 @@
         <x:v>0.4936708860759494</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2221,7 +2221,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="C12" s="19" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D12" s="19" t="n">
         <x:v>10</x:v>
@@ -2234,7 +2234,7 @@
         <x:v>0.42857142857142855</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2242,23 +2242,23 @@
         <x:v>Arquitectura</x:v>
       </x:c>
       <x:c r="B13" s="19" t="n">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C13" s="19" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D13" s="19" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E13" s="19" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F13" s="20" t="n">
         <x:f>IF(B13=0,"",E13/B13)</x:f>
-        <x:v>0.4444444444444444</x:v>
+        <x:v>0.4318181818181818</x:v>
       </x:c>
       <x:c r="G13" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2282,7 +2282,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2306,7 +2306,7 @@
         <x:v>0.38636363636363635</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2330,7 +2330,7 @@
         <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2344,17 +2344,17 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="D17" s="19" t="n">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E17" s="19" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F17" s="20" t="n">
         <x:f>IF(B17=0,"",E17/B17)</x:f>
-        <x:v>0.576271186440678</x:v>
+        <x:v>0.5932203389830508</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2365,10 +2365,10 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="C18" s="19" t="n">
-        <x:v>47</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D18" s="19" t="n">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E18" s="19" t="n">
         <x:v>35</x:v>
@@ -2378,7 +2378,7 @@
         <x:v>0.5303030303030303</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2386,7 +2386,7 @@
         <x:v>Contaduría Pública</x:v>
       </x:c>
       <x:c r="B19" s="19" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C19" s="19" t="n">
         <x:v>36</x:v>
@@ -2399,10 +2399,10 @@
       </x:c>
       <x:c r="F19" s="20" t="n">
         <x:f>IF(B19=0,"",E19/B19)</x:f>
-        <x:v>0.5471698113207547</x:v>
+        <x:v>0.5370370370370371</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2426,7 +2426,7 @@
         <x:v>0.5647058823529412</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2450,7 +2450,7 @@
         <x:v>0.52</x:v>
       </x:c>
       <x:c r="G21" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2474,7 +2474,7 @@
         <x:v>0.7346938775510204</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2498,7 +2498,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2522,7 +2522,7 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2533,7 +2533,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="C25" s="19" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D25" s="19" t="n">
         <x:v>30</x:v>
@@ -2546,7 +2546,7 @@
         <x:v>0.6410256410256411</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2554,7 +2554,7 @@
         <x:v>Técnico en Entrenamiento Deportivo</x:v>
       </x:c>
       <x:c r="B26" s="19" t="n">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C26" s="19" t="n">
         <x:v>18</x:v>
@@ -2567,10 +2567,10 @@
       </x:c>
       <x:c r="F26" s="20" t="n">
         <x:f>IF(B26=0,"",E26/B26)</x:f>
-        <x:v>0.5384615384615384</x:v>
+        <x:v>0.5185185185185185</x:v>
       </x:c>
       <x:c r="G26" t="str">
-        <x:v>EINR41 PS + RC · 19-08-2026</x:v>
+        <x:v>EINR41 PS + RC · 21-08-2026</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>